<commit_message>
fix: padronizacao da categoria Estocaveis e correcoes gerais
</commit_message>
<xml_diff>
--- a/Modelo_Importacao_GOM.xlsx
+++ b/Modelo_Importacao_GOM.xlsx
@@ -425,7 +425,7 @@
         <v>Arroz 5kg</v>
       </c>
       <c r="B2" t="str">
-        <v>ESTOCAVEIS</v>
+        <v>Estocáveis</v>
       </c>
       <c r="C2" t="str">
         <v>UN</v>
@@ -445,7 +445,7 @@
         <v>Feijão 1kg</v>
       </c>
       <c r="B3" t="str">
-        <v>ESTOCAVEIS</v>
+        <v>Estocáveis</v>
       </c>
       <c r="C3" t="str">
         <v>UN</v>
@@ -499,10 +499,10 @@
         <v>Arroz 5kg</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-07</v>
+        <v>2026-05-25</v>
       </c>
       <c r="C2" t="str">
-        <v>ESTOCAVEIS</v>
+        <v>Estocáveis</v>
       </c>
       <c r="D2" t="str">
         <v>UN</v>
@@ -522,10 +522,10 @@
         <v>Feijão 1kg</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-07</v>
+        <v>2026-05-25</v>
       </c>
       <c r="C3" t="str">
-        <v>ESTOCAVEIS</v>
+        <v>Estocáveis</v>
       </c>
       <c r="D3" t="str">
         <v>UN</v>

</xml_diff>

<commit_message>
Ajusta importacao de romaneio ao modelo
</commit_message>
<xml_diff>
--- a/Modelo_Importacao_GOM.xlsx
+++ b/Modelo_Importacao_GOM.xlsx
@@ -473,36 +473,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>PRODUTO</v>
+        <v>tipo</v>
       </c>
       <c r="B1" t="str">
-        <v>DATA</v>
+        <v>Depósito</v>
       </c>
       <c r="C1" t="str">
-        <v>CATEGORIA</v>
+        <v>produto</v>
       </c>
       <c r="D1" t="str">
-        <v>UND</v>
+        <v>und</v>
       </c>
       <c r="E1" t="str">
-        <v>QTD</v>
+        <v>qtd</v>
       </c>
       <c r="F1" t="str">
-        <v>DESTINO</v>
+        <v>Municipio</v>
       </c>
       <c r="G1" t="str">
-        <v>TIPO</v>
+        <v>data</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>SAIDA</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Depósito-Grupo OM</v>
+      </c>
+      <c r="C2" t="str">
         <v>Arroz 5kg</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-05-25</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Estocáveis</v>
       </c>
       <c r="D2" t="str">
         <v>UN</v>
@@ -514,18 +514,18 @@
         <v>Cozinha Central</v>
       </c>
       <c r="G2" t="str">
-        <v>SAIDA</v>
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>SAIDA</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Depósito-Grupo OM</v>
+      </c>
+      <c r="C3" t="str">
         <v>Feijão 1kg</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-05-25</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Estocáveis</v>
       </c>
       <c r="D3" t="str">
         <v>UN</v>
@@ -537,7 +537,7 @@
         <v>Doação</v>
       </c>
       <c r="G3" t="str">
-        <v>SAIDA</v>
+        <v>2026-07-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>